<commit_message>
feat(table): Luban gen pipeline working (gen scripts, __tables__/__beans__/__enums__ columns, tableImporter off, class->category)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#Action.xlsx
+++ b/table/Datas/#Action.xlsx
@@ -439,7 +439,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>class</t>
+          <t>category</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>class</t>
+          <t>category</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">

</xml_diff>